<commit_message>
Fix xlsx number formats, find's no-.git climb, and doc comment
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoUimiTUjEnP3nZA74hpFQ
</commit_message>
<xml_diff>
--- a/apply-design-system/examples/salari-test/sample.xlsx
+++ b/apply-design-system/examples/salari-test/sample.xlsx
@@ -9,9 +9,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.##"/>
-  </numFmts>
   <fonts count="5">
     <font>
       <sz val="11"/>
@@ -90,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -103,13 +100,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -200,36 +203,36 @@
       <c r="F4" s="4">
         <v>0</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="5">
         <v>4200.0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Placeholder A</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">A-102</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">9 x 12</t>
         </is>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="7">
         <v>7</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="7">
         <v>2</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="7">
         <v>1</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="8">
         <v>6150.5</v>
       </c>
     </row>
@@ -258,36 +261,36 @@
       <c r="F6" s="4">
         <v>0</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="5">
         <v>2875.0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Placeholder B</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">B-202</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">10 x 14</t>
         </is>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="7">
         <v>4</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="7">
         <v>3</v>
       </c>
-      <c r="F7" s="6">
-        <v>0</v>
-      </c>
-      <c r="G7" s="6">
+      <c r="F7" s="7">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
         <v>9400.0</v>
       </c>
     </row>
@@ -316,36 +319,36 @@
       <c r="F8" s="4">
         <v>2</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="5">
         <v>3990.0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Placeholder C</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">C-302</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">12 x 15</t>
         </is>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="7">
         <v>2</v>
       </c>
-      <c r="E9" s="6">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6">
+      <c r="E9" s="7">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7">
         <v>2</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="8">
         <v>12800.0</v>
       </c>
     </row>

</xml_diff>